<commit_message>
latest results based on simulated data uploaded
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Table_S1/g_output/D6_Table_S1_attrition_DPP4i.xlsx
+++ b/i_test/test_D6_Table_S1/g_output/D6_Table_S1_attrition_DPP4i.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -369,7 +369,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Totale popolazione in studio</t>
+          <t>Soggetti con almeno un farmaco nella storia e un observation period che overlappa lo study period</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -381,60 +381,120 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Totale soggetti registrati in anagrafe sanitaria al 1 gennaio di ogni anno tra 2016 e 2025</t>
+          <t>Totale soggetti registrati in anagrafe sanitaria per almeno un giorno tra il 01/01/2016 e il 31/12/2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.428 (28,6%)</t>
+          <t>4.002 (80,0%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Soggetti con una finestra di osservazione</t>
+          <t>Soggetti con un periodo di osservazione</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4.315 (86,3%)</t>
+          <t>4.000 (80,0%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Soggetti con almeno 2 anni di osservazione precedenti alla data di ingresso nella coorte di studio</t>
+          <t>Soggetti con un periodo di osservazione coincidente con il periodo di studio</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4.474 (89,5%)</t>
+          <t>4.034 (80,7%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Soggetti con prima dispensazione di farmaci di interesse nel periodo gen2016 - dic2025</t>
+          <t>Soggetti 18+ in almeno un giorno durante il periodo di studio</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.975 (79,5%)</t>
+          <t>4.010 (80,2%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Soggetti incidenti</t>
+          <t>Soggetti con almeno una dispensazione del farmaco di interesse nell’istanza</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.952 (59,0%)</t>
+          <t>3.976 (79,5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Soggetti con almeno una dispensazione del farmaco di interesse nel periodo di studio</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4.041 (80,8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Soggetti con almeno 2 anni di osservazione precedenti alla prima data di dispensazione del farmaco di interesse durante il periodo di studio (data indice)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4.015 (80,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Soggetti con ASL registrata alla data indice</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4.042 (80,8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Soggetti con nessuna dispensazione del farmaco di interesse nei due anni precedenti la data indice</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>437 (8,7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Totale soggetti inclusi nella coorte di studio</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>842 (16,8%)</t>
         </is>
       </c>
     </row>

</xml_diff>